<commit_message>
Add project 4 and 5
</commit_message>
<xml_diff>
--- a/projects/Formating.xlsx
+++ b/projects/Formating.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\T Irvin Pineda\Desktop\5 PROYECTOS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\T Irvin Pineda\Desktop\5 PROYECTOS\Excel-Simulator\projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A9A20B1-218D-4E70-8376-0247D8940022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{608245C8-DA2C-4F7F-860B-B2B6193E7914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="904" xr2:uid="{C5C32001-8B8D-4091-9E32-635000D0549A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="904" activeTab="2" xr2:uid="{C5C32001-8B8D-4091-9E32-635000D0549A}"/>
   </bookViews>
   <sheets>
     <sheet name="Ciberjuegos" sheetId="10" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="160">
   <si>
     <t>Año</t>
   </si>
@@ -531,25 +531,13 @@
   <si>
     <t>Total Sales</t>
   </si>
-  <si>
-    <t>Row Labels</t>
-  </si>
-  <si>
-    <t>Grand Total</t>
-  </si>
-  <si>
-    <t>Jun</t>
-  </si>
-  <si>
-    <t>Jul</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+    <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -628,7 +616,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -736,17 +724,124 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFABABAB"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFABABAB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFABABAB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFABABAB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFABABAB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFABABAB"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFABABAB"/>
+      </right>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFABABAB"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFABABAB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFABABAB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFABABAB"/>
+      </right>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFABABAB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -754,11 +849,11 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -766,6 +861,15 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
@@ -1139,7 +1243,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="165" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+      <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor theme="4" tint="0.79998168889431442"/>
@@ -1382,7 +1486,7 @@
     <worksheetSource name="Ventas_Videojuegos"/>
   </cacheSource>
   <cacheFields count="11">
-    <cacheField name="Año" numFmtId="165">
+    <cacheField name="Año" numFmtId="164">
       <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2022-06-02T00:00:00" maxDate="2022-07-09T00:00:00" count="37">
         <d v="2022-06-28T00:00:00"/>
         <d v="2022-06-07T00:00:00"/>
@@ -60645,8 +60749,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8893443A-6B87-4A2A-AE95-140F59CAB6CE}" name="TablaDinámica3" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:A6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8893443A-6B87-4A2A-AE95-140F59CAB6CE}" name="TablaDinámica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:C20" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
   <pivotFields count="11">
     <pivotField showAll="0">
       <items count="38">
@@ -64496,7 +64600,7 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
+    <pivotField showAll="0">
       <items count="369">
         <item sd="0" x="0"/>
         <item sd="0" x="1"/>
@@ -64869,7 +64973,7 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField axis="axisRow" showAll="0">
+    <pivotField showAll="0">
       <items count="15">
         <item sd="0" x="0"/>
         <item sd="0" x="1"/>
@@ -64889,24 +64993,6 @@
       </items>
     </pivotField>
   </pivotFields>
-  <rowFields count="2">
-    <field x="10"/>
-    <field x="9"/>
-  </rowFields>
-  <rowItems count="3">
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -65268,3024 +65354,3024 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="14"/>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="5" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="8">
+      <c r="A5" s="6">
         <v>44740</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="7">
         <v>29.02</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="7">
         <v>3.77</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="7">
         <v>8.4600000000000009</v>
       </c>
-      <c r="I5" s="10">
+      <c r="I5" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>12.23</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="11">
+      <c r="A6" s="9">
         <v>44719</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="1">
         <v>3.58</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="1">
         <v>6.81</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="1">
         <v>0.77</v>
       </c>
-      <c r="I6" s="10">
+      <c r="I6" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>7.58</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="8">
+      <c r="A7" s="6">
         <v>44742</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="7">
         <v>12.88</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="7">
         <v>3.79</v>
       </c>
-      <c r="H7" s="9">
+      <c r="H7" s="7">
         <v>3.31</v>
       </c>
-      <c r="I7" s="10">
+      <c r="I7" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>7.1</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="11">
+      <c r="A8" s="9">
         <v>44743</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="1">
         <v>11.01</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="1">
         <v>3.28</v>
       </c>
-      <c r="H8" s="3">
+      <c r="H8" s="1">
         <v>2.96</v>
       </c>
-      <c r="I8" s="10">
+      <c r="I8" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>6.24</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="8">
+      <c r="A9" s="6">
         <v>44730</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="7">
         <v>8.89</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="7">
         <v>10.220000000000001</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="7">
         <v>1</v>
       </c>
-      <c r="I9" s="10">
+      <c r="I9" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>11.22</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="11">
+      <c r="A10" s="9">
         <v>44723</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="1">
         <v>2.2599999999999998</v>
       </c>
-      <c r="G10" s="3">
+      <c r="G10" s="1">
         <v>4.22</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="1">
         <v>0.57999999999999996</v>
       </c>
-      <c r="I10" s="10">
+      <c r="I10" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>4.8</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="8">
+      <c r="A11" s="6">
         <v>44740</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F11" s="9">
+      <c r="F11" s="7">
         <v>9.23</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="7">
         <v>6.5</v>
       </c>
-      <c r="H11" s="9">
+      <c r="H11" s="7">
         <v>2.9</v>
       </c>
-      <c r="I11" s="10">
+      <c r="I11" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>9.4</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="11">
+      <c r="A12" s="9">
         <v>44740</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="1">
         <v>9.1999999999999993</v>
       </c>
-      <c r="G12" s="3">
+      <c r="G12" s="1">
         <v>2.93</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="1">
         <v>2.85</v>
       </c>
-      <c r="I12" s="10">
+      <c r="I12" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>5.78</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="8">
+      <c r="A13" s="6">
         <v>44743</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F13" s="9">
+      <c r="F13" s="7">
         <v>7.06</v>
       </c>
-      <c r="G13" s="9">
+      <c r="G13" s="7">
         <v>4.7</v>
       </c>
-      <c r="H13" s="9">
+      <c r="H13" s="7">
         <v>2.2599999999999998</v>
       </c>
-      <c r="I13" s="10">
+      <c r="I13" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>6.96</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="11">
+      <c r="A14" s="9">
         <v>44718</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="1">
         <v>0.63</v>
       </c>
-      <c r="G14" s="3">
+      <c r="G14" s="1">
         <v>0.28000000000000003</v>
       </c>
-      <c r="H14" s="3">
+      <c r="H14" s="1">
         <v>0.47</v>
       </c>
-      <c r="I14" s="10">
+      <c r="I14" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>0.75</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="8">
+      <c r="A15" s="6">
         <v>44739</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F15" s="9">
+      <c r="F15" s="7">
         <v>11</v>
       </c>
-      <c r="G15" s="9">
+      <c r="G15" s="7">
         <v>1.93</v>
       </c>
-      <c r="H15" s="9">
+      <c r="H15" s="7">
         <v>2.75</v>
       </c>
-      <c r="I15" s="10">
+      <c r="I15" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>4.68</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="11">
+      <c r="A16" s="9">
         <v>44739</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F16" s="3">
+      <c r="F16" s="1">
         <v>7.57</v>
       </c>
-      <c r="G16" s="3">
+      <c r="G16" s="1">
         <v>4.13</v>
       </c>
-      <c r="H16" s="3">
+      <c r="H16" s="1">
         <v>1.92</v>
       </c>
-      <c r="I16" s="10">
+      <c r="I16" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>6.05</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="8">
+      <c r="A17" s="6">
         <v>44733</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F17" s="9">
+      <c r="F17" s="7">
         <v>6.18</v>
       </c>
-      <c r="G17" s="9">
+      <c r="G17" s="7">
         <v>7.2</v>
       </c>
-      <c r="H17" s="9">
+      <c r="H17" s="7">
         <v>0.71</v>
       </c>
-      <c r="I17" s="10">
+      <c r="I17" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>7.91</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="11">
+      <c r="A18" s="9">
         <v>44741</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F18" s="3">
+      <c r="F18" s="1">
         <v>8.0299999999999994</v>
       </c>
-      <c r="G18" s="3">
+      <c r="G18" s="1">
         <v>3.6</v>
       </c>
-      <c r="H18" s="3">
+      <c r="H18" s="1">
         <v>2.15</v>
       </c>
-      <c r="I18" s="10">
+      <c r="I18" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>5.75</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="8">
+      <c r="A19" s="6">
         <v>44743</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="E19" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F19" s="9">
+      <c r="F19" s="7">
         <v>8.59</v>
       </c>
-      <c r="G19" s="9">
+      <c r="G19" s="7">
         <v>2.5299999999999998</v>
       </c>
-      <c r="H19" s="9">
+      <c r="H19" s="7">
         <v>1.79</v>
       </c>
-      <c r="I19" s="10">
+      <c r="I19" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>4.32</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="11">
+      <c r="A20" s="9">
         <v>44744</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F20" s="3">
+      <c r="F20" s="1">
         <v>4.9400000000000004</v>
       </c>
-      <c r="G20" s="3">
+      <c r="G20" s="1">
         <v>0.24</v>
       </c>
-      <c r="H20" s="3">
+      <c r="H20" s="1">
         <v>1.67</v>
       </c>
-      <c r="I20" s="10">
+      <c r="I20" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.91</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="8">
+      <c r="A21" s="6">
         <v>44747</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D21" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="E21" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="F21" s="9">
+      <c r="F21" s="7">
         <v>9.27</v>
       </c>
-      <c r="G21" s="9">
+      <c r="G21" s="7">
         <v>0.97</v>
       </c>
-      <c r="H21" s="9">
+      <c r="H21" s="7">
         <v>4.1399999999999997</v>
       </c>
-      <c r="I21" s="10">
+      <c r="I21" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>5.1099999999999994</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="11">
+      <c r="A22" s="9">
         <v>44738</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F22" s="3">
+      <c r="F22" s="1">
         <v>0.4</v>
       </c>
-      <c r="G22" s="3">
+      <c r="G22" s="1">
         <v>0.41</v>
       </c>
-      <c r="H22" s="3">
+      <c r="H22" s="1">
         <v>10.57</v>
       </c>
-      <c r="I22" s="10">
+      <c r="I22" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>10.98</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="8">
+      <c r="A23" s="6">
         <v>44724</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="D23" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="E23" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F23" s="9">
+      <c r="F23" s="7">
         <v>3.75</v>
       </c>
-      <c r="G23" s="9">
+      <c r="G23" s="7">
         <v>3.54</v>
       </c>
-      <c r="H23" s="9">
+      <c r="H23" s="7">
         <v>0.55000000000000004</v>
       </c>
-      <c r="I23" s="10">
+      <c r="I23" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>4.09</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="11">
+      <c r="A24" s="9">
         <v>44739</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F24" s="3">
+      <c r="F24" s="1">
         <v>9.26</v>
       </c>
-      <c r="G24" s="3">
+      <c r="G24" s="1">
         <v>4.16</v>
       </c>
-      <c r="H24" s="3">
+      <c r="H24" s="1">
         <v>2.0499999999999998</v>
       </c>
-      <c r="I24" s="10">
+      <c r="I24" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>6.21</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="8">
+      <c r="A25" s="6">
         <v>44740</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="D25" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F25" s="9">
+      <c r="F25" s="7">
         <v>4.5199999999999996</v>
       </c>
-      <c r="G25" s="9">
+      <c r="G25" s="7">
         <v>6.04</v>
       </c>
-      <c r="H25" s="9">
+      <c r="H25" s="7">
         <v>1.37</v>
       </c>
-      <c r="I25" s="10">
+      <c r="I25" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>7.41</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="11">
+      <c r="A26" s="9">
         <v>44723</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="E26" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F26" s="3">
+      <c r="F26" s="1">
         <v>2.71</v>
       </c>
-      <c r="G26" s="3">
+      <c r="G26" s="1">
         <v>4.18</v>
       </c>
-      <c r="H26" s="3">
+      <c r="H26" s="1">
         <v>0.42</v>
       </c>
-      <c r="I26" s="10">
+      <c r="I26" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="8">
+      <c r="A27" s="6">
         <v>44722</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="D27" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="E27" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F27" s="9">
+      <c r="F27" s="7">
         <v>3.44</v>
       </c>
-      <c r="G27" s="9">
+      <c r="G27" s="7">
         <v>3.84</v>
       </c>
-      <c r="H27" s="9">
+      <c r="H27" s="7">
         <v>0.46</v>
       </c>
-      <c r="I27" s="10">
+      <c r="I27" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>4.3</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="11">
+      <c r="A28" s="9">
         <v>44747</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D28" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F28" s="3">
+      <c r="F28" s="1">
         <v>5.31</v>
       </c>
-      <c r="G28" s="3">
+      <c r="G28" s="1">
         <v>0.06</v>
       </c>
-      <c r="H28" s="3">
+      <c r="H28" s="1">
         <v>1.38</v>
       </c>
-      <c r="I28" s="10">
+      <c r="I28" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.44</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="8">
+      <c r="A29" s="6">
         <v>44736</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="B29" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="C29" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D29" s="9" t="s">
+      <c r="D29" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E29" s="9" t="s">
+      <c r="E29" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="F29" s="9">
+      <c r="F29" s="7">
         <v>5.49</v>
       </c>
-      <c r="G29" s="9">
+      <c r="G29" s="7">
         <v>0.47</v>
       </c>
-      <c r="H29" s="9">
+      <c r="H29" s="7">
         <v>1.78</v>
       </c>
-      <c r="I29" s="10">
+      <c r="I29" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.25</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="11">
+      <c r="A30" s="9">
         <v>44736</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="E30" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F30" s="3">
+      <c r="F30" s="1">
         <v>3.9</v>
       </c>
-      <c r="G30" s="3">
+      <c r="G30" s="1">
         <v>5.38</v>
       </c>
-      <c r="H30" s="3">
+      <c r="H30" s="1">
         <v>0.5</v>
       </c>
-      <c r="I30" s="10">
+      <c r="I30" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>5.88</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="8">
+      <c r="A31" s="6">
         <v>44744</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="B31" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D31" s="9" t="s">
+      <c r="D31" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E31" s="9" t="s">
+      <c r="E31" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F31" s="9">
+      <c r="F31" s="7">
         <v>3.28</v>
       </c>
-      <c r="G31" s="9">
+      <c r="G31" s="7">
         <v>5.65</v>
       </c>
-      <c r="H31" s="9">
+      <c r="H31" s="7">
         <v>0.82</v>
       </c>
-      <c r="I31" s="10">
+      <c r="I31" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>6.4700000000000006</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="11">
+      <c r="A32" s="9">
         <v>44739</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="D32" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="E32" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F32" s="3">
+      <c r="F32" s="1">
         <v>5.36</v>
       </c>
-      <c r="G32" s="3">
+      <c r="G32" s="1">
         <v>5.32</v>
       </c>
-      <c r="H32" s="3">
+      <c r="H32" s="1">
         <v>1.18</v>
       </c>
-      <c r="I32" s="10">
+      <c r="I32" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>6.5</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="8">
+      <c r="A33" s="6">
         <v>44735</v>
       </c>
-      <c r="B33" s="9" t="s">
+      <c r="B33" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="C33" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D33" s="9" t="s">
+      <c r="D33" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E33" s="9" t="s">
+      <c r="E33" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F33" s="9">
+      <c r="F33" s="7">
         <v>5.09</v>
       </c>
-      <c r="G33" s="9">
+      <c r="G33" s="7">
         <v>1.87</v>
       </c>
-      <c r="H33" s="9">
+      <c r="H33" s="7">
         <v>1.1599999999999999</v>
       </c>
-      <c r="I33" s="10">
+      <c r="I33" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>3.0300000000000002</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="11">
+      <c r="A34" s="9">
         <v>44745</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="D34" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="E34" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F34" s="3">
+      <c r="F34" s="1">
         <v>4.28</v>
       </c>
-      <c r="G34" s="3">
+      <c r="G34" s="1">
         <v>0.13</v>
       </c>
-      <c r="H34" s="3">
+      <c r="H34" s="1">
         <v>1.32</v>
       </c>
-      <c r="I34" s="10">
+      <c r="I34" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.4500000000000002</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="8">
+      <c r="A35" s="6">
         <v>44732</v>
       </c>
-      <c r="B35" s="9" t="s">
+      <c r="B35" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D35" s="9" t="s">
+      <c r="D35" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E35" s="9" t="s">
+      <c r="E35" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F35" s="9">
+      <c r="F35" s="7">
         <v>5.04</v>
       </c>
-      <c r="G35" s="9">
+      <c r="G35" s="7">
         <v>3.12</v>
       </c>
-      <c r="H35" s="9">
+      <c r="H35" s="7">
         <v>0.59</v>
       </c>
-      <c r="I35" s="10">
+      <c r="I35" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>3.71</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="11">
+      <c r="A36" s="9">
         <v>44744</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B36" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="D36" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="E36" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F36" s="3">
+      <c r="F36" s="1">
         <v>3.73</v>
       </c>
-      <c r="G36" s="3">
+      <c r="G36" s="1">
         <v>0.11</v>
       </c>
-      <c r="H36" s="3">
+      <c r="H36" s="1">
         <v>1.1299999999999999</v>
       </c>
-      <c r="I36" s="10">
+      <c r="I36" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.24</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="8">
+      <c r="A37" s="6">
         <v>44747</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="B37" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="C37" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="D37" s="9" t="s">
+      <c r="D37" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E37" s="9" t="s">
+      <c r="E37" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F37" s="9">
+      <c r="F37" s="7">
         <v>4.05</v>
       </c>
-      <c r="G37" s="9">
+      <c r="G37" s="7">
         <v>4.34</v>
       </c>
-      <c r="H37" s="9">
+      <c r="H37" s="7">
         <v>0.79</v>
       </c>
-      <c r="I37" s="10">
+      <c r="I37" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>5.13</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="11">
+      <c r="A38" s="9">
         <v>44749</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="B38" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="C38" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="D38" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="E38" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F38" s="3">
+      <c r="F38" s="1">
         <v>5.81</v>
       </c>
-      <c r="G38" s="3">
+      <c r="G38" s="1">
         <v>0.35</v>
       </c>
-      <c r="H38" s="3">
+      <c r="H38" s="1">
         <v>2.31</v>
       </c>
-      <c r="I38" s="10">
+      <c r="I38" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.66</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="8">
+      <c r="A39" s="6">
         <v>44746</v>
       </c>
-      <c r="B39" s="9" t="s">
+      <c r="B39" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="C39" s="9" t="s">
+      <c r="C39" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D39" s="9" t="s">
+      <c r="D39" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E39" s="9" t="s">
+      <c r="E39" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F39" s="9">
+      <c r="F39" s="7">
         <v>5.88</v>
       </c>
-      <c r="G39" s="9">
+      <c r="G39" s="7">
         <v>0.65</v>
       </c>
-      <c r="H39" s="9">
+      <c r="H39" s="7">
         <v>2.52</v>
       </c>
-      <c r="I39" s="10">
+      <c r="I39" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>3.17</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="11">
+      <c r="A40" s="9">
         <v>44746</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="B40" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="C40" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="D40" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E40" s="3" t="s">
+      <c r="E40" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F40" s="3">
+      <c r="F40" s="1">
         <v>4.3</v>
       </c>
-      <c r="G40" s="3">
+      <c r="G40" s="1">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="H40" s="3">
+      <c r="H40" s="1">
         <v>1.1200000000000001</v>
       </c>
-      <c r="I40" s="10">
+      <c r="I40" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.1900000000000002</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="8">
+      <c r="A41" s="6">
         <v>44743</v>
       </c>
-      <c r="B41" s="9" t="s">
+      <c r="B41" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C41" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D41" s="9" t="s">
+      <c r="D41" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E41" s="9" t="s">
+      <c r="E41" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F41" s="9">
+      <c r="F41" s="7">
         <v>3.63</v>
       </c>
-      <c r="G41" s="9">
+      <c r="G41" s="7">
         <v>0.08</v>
       </c>
-      <c r="H41" s="9">
+      <c r="H41" s="7">
         <v>1.29</v>
       </c>
-      <c r="I41" s="10">
+      <c r="I41" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.37</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="11">
+      <c r="A42" s="9">
         <v>44745</v>
       </c>
-      <c r="B42" s="3" t="s">
+      <c r="B42" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C42" s="3" t="s">
+      <c r="C42" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D42" s="3" t="s">
+      <c r="D42" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E42" s="3" t="s">
+      <c r="E42" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F42" s="3">
+      <c r="F42" s="1">
         <v>5.82</v>
       </c>
-      <c r="G42" s="3">
+      <c r="G42" s="1">
         <v>0.49</v>
       </c>
-      <c r="H42" s="3">
+      <c r="H42" s="1">
         <v>1.62</v>
       </c>
-      <c r="I42" s="10">
+      <c r="I42" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.1100000000000003</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="8">
+      <c r="A43" s="6">
         <v>44735</v>
       </c>
-      <c r="B43" s="9" t="s">
+      <c r="B43" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="C43" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D43" s="9" t="s">
+      <c r="D43" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E43" s="9" t="s">
+      <c r="E43" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="F43" s="9">
+      <c r="F43" s="7">
         <v>4.51</v>
       </c>
-      <c r="G43" s="9">
+      <c r="G43" s="7">
         <v>0.3</v>
       </c>
-      <c r="H43" s="9">
+      <c r="H43" s="7">
         <v>1.3</v>
       </c>
-      <c r="I43" s="10">
+      <c r="I43" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.6</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="11">
+      <c r="A44" s="9">
         <v>44742</v>
       </c>
-      <c r="B44" s="3" t="s">
+      <c r="B44" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C44" s="3" t="s">
+      <c r="C44" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D44" s="3" t="s">
+      <c r="D44" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E44" s="3" t="s">
+      <c r="E44" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F44" s="3">
+      <c r="F44" s="1">
         <v>2.61</v>
       </c>
-      <c r="G44" s="3">
+      <c r="G44" s="1">
         <v>2.66</v>
       </c>
-      <c r="H44" s="3">
+      <c r="H44" s="1">
         <v>1.02</v>
       </c>
-      <c r="I44" s="10">
+      <c r="I44" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>3.68</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="8">
+      <c r="A45" s="6">
         <v>44744</v>
       </c>
-      <c r="B45" s="9" t="s">
+      <c r="B45" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C45" s="9" t="s">
+      <c r="C45" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D45" s="9" t="s">
+      <c r="D45" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E45" s="9" t="s">
+      <c r="E45" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F45" s="9">
+      <c r="F45" s="7">
         <v>4.4400000000000004</v>
       </c>
-      <c r="G45" s="9">
+      <c r="G45" s="7">
         <v>0.48</v>
       </c>
-      <c r="H45" s="9">
+      <c r="H45" s="7">
         <v>1.83</v>
       </c>
-      <c r="I45" s="10">
+      <c r="I45" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.31</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="11">
+      <c r="A46" s="9">
         <v>44739</v>
       </c>
-      <c r="B46" s="3" t="s">
+      <c r="B46" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C46" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D46" s="3" t="s">
+      <c r="D46" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E46" s="3" t="s">
+      <c r="E46" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F46" s="3">
+      <c r="F46" s="1">
         <v>3.52</v>
       </c>
-      <c r="G46" s="3">
+      <c r="G46" s="1">
         <v>5.33</v>
       </c>
-      <c r="H46" s="3">
+      <c r="H46" s="1">
         <v>0.88</v>
       </c>
-      <c r="I46" s="10">
+      <c r="I46" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>6.21</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="8">
+      <c r="A47" s="6">
         <v>44745</v>
       </c>
-      <c r="B47" s="9" t="s">
+      <c r="B47" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C47" s="9" t="s">
+      <c r="C47" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="D47" s="9" t="s">
+      <c r="D47" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E47" s="9" t="s">
+      <c r="E47" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F47" s="9">
+      <c r="F47" s="7">
         <v>3.91</v>
       </c>
-      <c r="G47" s="9">
+      <c r="G47" s="7">
         <v>2.67</v>
       </c>
-      <c r="H47" s="9">
+      <c r="H47" s="7">
         <v>0.89</v>
       </c>
-      <c r="I47" s="10">
+      <c r="I47" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>3.56</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="11">
+      <c r="A48" s="9">
         <v>44741</v>
       </c>
-      <c r="B48" s="3" t="s">
+      <c r="B48" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C48" s="3" t="s">
+      <c r="C48" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D48" s="3" t="s">
+      <c r="D48" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E48" s="3" t="s">
+      <c r="E48" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F48" s="3">
+      <c r="F48" s="1">
         <v>2.83</v>
       </c>
-      <c r="G48" s="3">
+      <c r="G48" s="1">
         <v>0.13</v>
       </c>
-      <c r="H48" s="3">
+      <c r="H48" s="1">
         <v>1.21</v>
       </c>
-      <c r="I48" s="10">
+      <c r="I48" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.3399999999999999</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="8">
+      <c r="A49" s="6">
         <v>44748</v>
       </c>
-      <c r="B49" s="9" t="s">
+      <c r="B49" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="C49" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="D49" s="9" t="s">
+      <c r="D49" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E49" s="9" t="s">
+      <c r="E49" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="F49" s="9">
+      <c r="F49" s="7">
         <v>5.81</v>
       </c>
-      <c r="G49" s="9">
+      <c r="G49" s="7">
         <v>0.36</v>
       </c>
-      <c r="H49" s="9">
+      <c r="H49" s="7">
         <v>2.02</v>
       </c>
-      <c r="I49" s="10">
+      <c r="I49" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.38</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A50" s="11">
+      <c r="A50" s="9">
         <v>44743</v>
       </c>
-      <c r="B50" s="3" t="s">
+      <c r="B50" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C50" s="3" t="s">
+      <c r="C50" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D50" s="3" t="s">
+      <c r="D50" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E50" s="3" t="s">
+      <c r="E50" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F50" s="3">
+      <c r="F50" s="1">
         <v>2.77</v>
       </c>
-      <c r="G50" s="3">
+      <c r="G50" s="1">
         <v>3.96</v>
       </c>
-      <c r="H50" s="3">
+      <c r="H50" s="1">
         <v>0.77</v>
       </c>
-      <c r="I50" s="10">
+      <c r="I50" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>4.7300000000000004</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A51" s="8">
+      <c r="A51" s="6">
         <v>44730</v>
       </c>
-      <c r="B51" s="9" t="s">
+      <c r="B51" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="C51" s="9" t="s">
+      <c r="C51" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="D51" s="9" t="s">
+      <c r="D51" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E51" s="9" t="s">
+      <c r="E51" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F51" s="9">
+      <c r="F51" s="7">
         <v>2.85</v>
       </c>
-      <c r="G51" s="9">
+      <c r="G51" s="7">
         <v>1.91</v>
       </c>
-      <c r="H51" s="9">
+      <c r="H51" s="7">
         <v>0.23</v>
       </c>
-      <c r="I51" s="10">
+      <c r="I51" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.14</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="11">
+      <c r="A52" s="9">
         <v>44738</v>
       </c>
-      <c r="B52" s="3" t="s">
+      <c r="B52" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C52" s="3" t="s">
+      <c r="C52" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D52" s="3" t="s">
+      <c r="D52" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E52" s="3" t="s">
+      <c r="E52" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F52" s="3">
+      <c r="F52" s="1">
         <v>0.01</v>
       </c>
-      <c r="G52" s="3">
+      <c r="G52" s="1">
         <v>1.1000000000000001</v>
       </c>
-      <c r="H52" s="3">
+      <c r="H52" s="1">
         <v>7.53</v>
       </c>
-      <c r="I52" s="10">
+      <c r="I52" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>8.6300000000000008</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A53" s="8">
+      <c r="A53" s="6">
         <v>44741</v>
       </c>
-      <c r="B53" s="9" t="s">
+      <c r="B53" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C53" s="9" t="s">
+      <c r="C53" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D53" s="9" t="s">
+      <c r="D53" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E53" s="9" t="s">
+      <c r="E53" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F53" s="9">
+      <c r="F53" s="7">
         <v>3.4</v>
       </c>
-      <c r="G53" s="9">
+      <c r="G53" s="7">
         <v>1.2</v>
       </c>
-      <c r="H53" s="9">
+      <c r="H53" s="7">
         <v>0.76</v>
       </c>
-      <c r="I53" s="10">
+      <c r="I53" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.96</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A54" s="11">
+      <c r="A54" s="9">
         <v>44748</v>
       </c>
-      <c r="B54" s="3" t="s">
+      <c r="B54" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C54" s="3" t="s">
+      <c r="C54" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D54" s="3" t="s">
+      <c r="D54" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E54" s="3" t="s">
+      <c r="E54" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F54" s="3">
+      <c r="F54" s="1">
         <v>3.37</v>
       </c>
-      <c r="G54" s="3">
+      <c r="G54" s="1">
         <v>3.08</v>
       </c>
-      <c r="H54" s="3">
+      <c r="H54" s="1">
         <v>0.65</v>
       </c>
-      <c r="I54" s="10">
+      <c r="I54" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>3.73</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A55" s="8">
+      <c r="A55" s="6">
         <v>44726</v>
       </c>
-      <c r="B55" s="9" t="s">
+      <c r="B55" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C55" s="9" t="s">
+      <c r="C55" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D55" s="9" t="s">
+      <c r="D55" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="E55" s="9" t="s">
+      <c r="E55" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F55" s="9">
+      <c r="F55" s="7">
         <v>2.04</v>
       </c>
-      <c r="G55" s="9">
+      <c r="G55" s="7">
         <v>2.69</v>
       </c>
-      <c r="H55" s="9">
+      <c r="H55" s="7">
         <v>0.28999999999999998</v>
       </c>
-      <c r="I55" s="10">
+      <c r="I55" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.98</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A56" s="11">
+      <c r="A56" s="9">
         <v>44742</v>
       </c>
-      <c r="B56" s="3" t="s">
+      <c r="B56" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C56" s="3" t="s">
+      <c r="C56" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D56" s="3" t="s">
+      <c r="D56" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E56" s="3" t="s">
+      <c r="E56" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F56" s="3">
+      <c r="F56" s="1">
         <v>3.1</v>
       </c>
-      <c r="G56" s="3">
+      <c r="G56" s="1">
         <v>0.14000000000000001</v>
       </c>
-      <c r="H56" s="3">
+      <c r="H56" s="1">
         <v>1.03</v>
       </c>
-      <c r="I56" s="10">
+      <c r="I56" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.17</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A57" s="8">
+      <c r="A57" s="6">
         <v>44731</v>
       </c>
-      <c r="B57" s="9" t="s">
+      <c r="B57" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C57" s="9" t="s">
+      <c r="C57" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D57" s="9" t="s">
+      <c r="D57" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E57" s="9" t="s">
+      <c r="E57" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F57" s="9">
+      <c r="F57" s="7">
         <v>3.87</v>
       </c>
-      <c r="G57" s="9">
+      <c r="G57" s="7">
         <v>2.54</v>
       </c>
-      <c r="H57" s="9">
+      <c r="H57" s="7">
         <v>0.52</v>
       </c>
-      <c r="I57" s="10">
+      <c r="I57" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>3.06</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A58" s="11">
+      <c r="A58" s="9">
         <v>44745</v>
       </c>
-      <c r="B58" s="3" t="s">
+      <c r="B58" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C58" s="3" t="s">
+      <c r="C58" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D58" s="3" t="s">
+      <c r="D58" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E58" s="3" t="s">
+      <c r="E58" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F58" s="3">
+      <c r="F58" s="1">
         <v>2.99</v>
       </c>
-      <c r="G58" s="3">
+      <c r="G58" s="1">
         <v>2.13</v>
       </c>
-      <c r="H58" s="3">
+      <c r="H58" s="1">
         <v>0.78</v>
       </c>
-      <c r="I58" s="10">
+      <c r="I58" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.91</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A59" s="8">
+      <c r="A59" s="6">
         <v>44744</v>
       </c>
-      <c r="B59" s="9" t="s">
+      <c r="B59" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="C59" s="9" t="s">
+      <c r="C59" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D59" s="9" t="s">
+      <c r="D59" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E59" s="9" t="s">
+      <c r="E59" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F59" s="9">
+      <c r="F59" s="7">
         <v>4.88</v>
       </c>
-      <c r="G59" s="9">
+      <c r="G59" s="7">
         <v>0.81</v>
       </c>
-      <c r="H59" s="9">
+      <c r="H59" s="7">
         <v>2.12</v>
       </c>
-      <c r="I59" s="10">
+      <c r="I59" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.93</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A60" s="11">
+      <c r="A60" s="9">
         <v>44743</v>
       </c>
-      <c r="B60" s="3" t="s">
+      <c r="B60" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C60" s="3" t="s">
+      <c r="C60" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D60" s="3" t="s">
+      <c r="D60" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E60" s="3" t="s">
+      <c r="E60" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F60" s="3">
+      <c r="F60" s="1">
         <v>3.69</v>
       </c>
-      <c r="G60" s="3">
+      <c r="G60" s="1">
         <v>0.38</v>
       </c>
-      <c r="H60" s="3">
+      <c r="H60" s="1">
         <v>1.63</v>
       </c>
-      <c r="I60" s="10">
+      <c r="I60" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.0099999999999998</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A61" s="8">
+      <c r="A61" s="6">
         <v>44742</v>
       </c>
-      <c r="B61" s="9" t="s">
+      <c r="B61" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C61" s="9" t="s">
+      <c r="C61" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D61" s="9" t="s">
+      <c r="D61" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E61" s="9" t="s">
+      <c r="E61" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="F61" s="9">
+      <c r="F61" s="7">
         <v>3.76</v>
       </c>
-      <c r="G61" s="9">
+      <c r="G61" s="7">
         <v>0.44</v>
       </c>
-      <c r="H61" s="9">
+      <c r="H61" s="7">
         <v>1.62</v>
       </c>
-      <c r="I61" s="10">
+      <c r="I61" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.06</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A62" s="11">
+      <c r="A62" s="9">
         <v>44727</v>
       </c>
-      <c r="B62" s="3" t="s">
+      <c r="B62" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C62" s="3" t="s">
+      <c r="C62" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D62" s="3" t="s">
+      <c r="D62" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E62" s="3" t="s">
+      <c r="E62" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F62" s="3">
+      <c r="F62" s="1">
         <v>2.15</v>
       </c>
-      <c r="G62" s="3">
+      <c r="G62" s="1">
         <v>2.12</v>
       </c>
-      <c r="H62" s="3">
+      <c r="H62" s="1">
         <v>0.28999999999999998</v>
       </c>
-      <c r="I62" s="10">
+      <c r="I62" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.41</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A63" s="8">
+      <c r="A63" s="6">
         <v>44738</v>
       </c>
-      <c r="B63" s="9" t="s">
+      <c r="B63" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C63" s="9" t="s">
+      <c r="C63" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D63" s="9" t="s">
+      <c r="D63" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E63" s="9" t="s">
+      <c r="E63" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F63" s="9">
+      <c r="F63" s="7">
         <v>2.65</v>
       </c>
-      <c r="G63" s="9">
+      <c r="G63" s="7">
         <v>3.15</v>
       </c>
-      <c r="H63" s="9">
+      <c r="H63" s="7">
         <v>0.35</v>
       </c>
-      <c r="I63" s="10">
+      <c r="I63" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>3.5</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A64" s="11">
+      <c r="A64" s="9">
         <v>44738</v>
       </c>
-      <c r="B64" s="3" t="s">
+      <c r="B64" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C64" s="3" t="s">
+      <c r="C64" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D64" s="3" t="s">
+      <c r="D64" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E64" s="3" t="s">
+      <c r="E64" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F64" s="3">
+      <c r="F64" s="1">
         <v>3.11</v>
       </c>
-      <c r="G64" s="3">
+      <c r="G64" s="1">
         <v>1.25</v>
       </c>
-      <c r="H64" s="3">
+      <c r="H64" s="1">
         <v>0.98</v>
       </c>
-      <c r="I64" s="10">
+      <c r="I64" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.23</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A65" s="8">
+      <c r="A65" s="6">
         <v>44745</v>
       </c>
-      <c r="B65" s="9" t="s">
+      <c r="B65" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="C65" s="9" t="s">
+      <c r="C65" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D65" s="9" t="s">
+      <c r="D65" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E65" s="9" t="s">
+      <c r="E65" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="F65" s="9">
+      <c r="F65" s="7">
         <v>3.15</v>
       </c>
-      <c r="G65" s="9">
+      <c r="G65" s="7">
         <v>0</v>
       </c>
-      <c r="H65" s="9">
+      <c r="H65" s="7">
         <v>1.07</v>
       </c>
-      <c r="I65" s="10">
+      <c r="I65" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.07</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A66" s="11">
+      <c r="A66" s="9">
         <v>44747</v>
       </c>
-      <c r="B66" s="3" t="s">
+      <c r="B66" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C66" s="3" t="s">
+      <c r="C66" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D66" s="3" t="s">
+      <c r="D66" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E66" s="3" t="s">
+      <c r="E66" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F66" s="3">
+      <c r="F66" s="1">
         <v>2.63</v>
       </c>
-      <c r="G66" s="3">
+      <c r="G66" s="1">
         <v>0.04</v>
       </c>
-      <c r="H66" s="3">
+      <c r="H66" s="1">
         <v>0.82</v>
       </c>
-      <c r="I66" s="10">
+      <c r="I66" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>0.86</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A67" s="8">
+      <c r="A67" s="6">
         <v>44744</v>
       </c>
-      <c r="B67" s="9" t="s">
+      <c r="B67" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="C67" s="9" t="s">
+      <c r="C67" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D67" s="9" t="s">
+      <c r="D67" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E67" s="9" t="s">
+      <c r="E67" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="F67" s="9">
+      <c r="F67" s="7">
         <v>1.98</v>
       </c>
-      <c r="G67" s="9">
+      <c r="G67" s="7">
         <v>0.08</v>
       </c>
-      <c r="H67" s="9">
+      <c r="H67" s="7">
         <v>0.78</v>
       </c>
-      <c r="I67" s="10">
+      <c r="I67" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>0.86</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A68" s="11">
+      <c r="A68" s="9">
         <v>44730</v>
       </c>
-      <c r="B68" s="3" t="s">
+      <c r="B68" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C68" s="3" t="s">
+      <c r="C68" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D68" s="3" t="s">
+      <c r="D68" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E68" s="3" t="s">
+      <c r="E68" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F68" s="3">
+      <c r="F68" s="1">
         <v>1.94</v>
       </c>
-      <c r="G68" s="3">
+      <c r="G68" s="1">
         <v>2.23</v>
       </c>
-      <c r="H68" s="3">
+      <c r="H68" s="1">
         <v>0.15</v>
       </c>
-      <c r="I68" s="10">
+      <c r="I68" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.38</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A69" s="8">
+      <c r="A69" s="6">
         <v>44746</v>
       </c>
-      <c r="B69" s="9" t="s">
+      <c r="B69" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="C69" s="9" t="s">
+      <c r="C69" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="D69" s="9" t="s">
+      <c r="D69" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E69" s="9" t="s">
+      <c r="E69" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F69" s="9">
+      <c r="F69" s="7">
         <v>3.07</v>
       </c>
-      <c r="G69" s="9">
+      <c r="G69" s="7">
         <v>2.4700000000000002</v>
       </c>
-      <c r="H69" s="9">
+      <c r="H69" s="7">
         <v>0.63</v>
       </c>
-      <c r="I69" s="10">
+      <c r="I69" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>3.1</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A70" s="11">
+      <c r="A70" s="9">
         <v>44746</v>
       </c>
-      <c r="B70" s="3" t="s">
+      <c r="B70" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C70" s="3" t="s">
+      <c r="C70" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D70" s="3" t="s">
+      <c r="D70" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E70" s="3" t="s">
+      <c r="E70" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F70" s="3">
+      <c r="F70" s="1">
         <v>2.36</v>
       </c>
-      <c r="G70" s="3">
+      <c r="G70" s="1">
         <v>0.04</v>
       </c>
-      <c r="H70" s="3">
+      <c r="H70" s="1">
         <v>0.73</v>
       </c>
-      <c r="I70" s="10">
+      <c r="I70" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>0.77</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A71" s="8">
+      <c r="A71" s="6">
         <v>44731</v>
       </c>
-      <c r="B71" s="9" t="s">
+      <c r="B71" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="C71" s="9" t="s">
+      <c r="C71" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D71" s="9" t="s">
+      <c r="D71" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E71" s="9" t="s">
+      <c r="E71" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F71" s="9">
+      <c r="F71" s="7">
         <v>2.4700000000000002</v>
       </c>
-      <c r="G71" s="9">
+      <c r="G71" s="7">
         <v>3.28</v>
       </c>
-      <c r="H71" s="9">
+      <c r="H71" s="7">
         <v>0.96</v>
       </c>
-      <c r="I71" s="10">
+      <c r="I71" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>4.24</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A72" s="11">
+      <c r="A72" s="9">
         <v>44747</v>
       </c>
-      <c r="B72" s="3" t="s">
+      <c r="B72" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C72" s="3" t="s">
+      <c r="C72" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D72" s="3" t="s">
+      <c r="D72" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E72" s="3" t="s">
+      <c r="E72" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F72" s="3">
+      <c r="F72" s="1">
         <v>3.73</v>
       </c>
-      <c r="G72" s="3">
+      <c r="G72" s="1">
         <v>0.38</v>
       </c>
-      <c r="H72" s="3">
+      <c r="H72" s="1">
         <v>1.38</v>
       </c>
-      <c r="I72" s="10">
+      <c r="I72" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.7599999999999998</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A73" s="8">
+      <c r="A73" s="6">
         <v>44744</v>
       </c>
-      <c r="B73" s="9" t="s">
+      <c r="B73" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="C73" s="9" t="s">
+      <c r="C73" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D73" s="9" t="s">
+      <c r="D73" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E73" s="9" t="s">
+      <c r="E73" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="F73" s="9">
+      <c r="F73" s="7">
         <v>2.89</v>
       </c>
-      <c r="G73" s="9">
+      <c r="G73" s="7">
         <v>0.01</v>
       </c>
-      <c r="H73" s="9">
+      <c r="H73" s="7">
         <v>0.78</v>
       </c>
-      <c r="I73" s="10">
+      <c r="I73" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>0.79</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A74" s="11">
+      <c r="A74" s="9">
         <v>44733</v>
       </c>
-      <c r="B74" s="3" t="s">
+      <c r="B74" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C74" s="3" t="s">
+      <c r="C74" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="D74" s="3" t="s">
+      <c r="D74" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E74" s="3" t="s">
+      <c r="E74" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F74" s="3">
+      <c r="F74" s="1">
         <v>3.42</v>
       </c>
-      <c r="G74" s="3">
+      <c r="G74" s="1">
         <v>1.69</v>
       </c>
-      <c r="H74" s="3">
+      <c r="H74" s="1">
         <v>0.5</v>
       </c>
-      <c r="I74" s="10">
+      <c r="I74" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.19</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A75" s="8">
+      <c r="A75" s="6">
         <v>44741</v>
       </c>
-      <c r="B75" s="9" t="s">
+      <c r="B75" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="C75" s="9" t="s">
+      <c r="C75" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D75" s="9" t="s">
+      <c r="D75" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E75" s="9" t="s">
+      <c r="E75" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F75" s="9">
+      <c r="F75" s="7">
         <v>2.38</v>
       </c>
-      <c r="G75" s="9">
+      <c r="G75" s="7">
         <v>0.13</v>
       </c>
-      <c r="H75" s="9">
+      <c r="H75" s="7">
         <v>0.9</v>
       </c>
-      <c r="I75" s="10">
+      <c r="I75" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.03</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A76" s="11">
+      <c r="A76" s="9">
         <v>44728</v>
       </c>
-      <c r="B76" s="3" t="s">
+      <c r="B76" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C76" s="3" t="s">
+      <c r="C76" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D76" s="3" t="s">
+      <c r="D76" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E76" s="3" t="s">
+      <c r="E76" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F76" s="3">
+      <c r="F76" s="1">
         <v>1.71</v>
       </c>
-      <c r="G76" s="3">
+      <c r="G76" s="1">
         <v>3</v>
       </c>
-      <c r="H76" s="3">
+      <c r="H76" s="1">
         <v>0.23</v>
       </c>
-      <c r="I76" s="10">
+      <c r="I76" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>3.23</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A77" s="8">
+      <c r="A77" s="6">
         <v>44747</v>
       </c>
-      <c r="B77" s="9" t="s">
+      <c r="B77" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="C77" s="9" t="s">
+      <c r="C77" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D77" s="9" t="s">
+      <c r="D77" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E77" s="9" t="s">
+      <c r="E77" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="F77" s="9">
+      <c r="F77" s="7">
         <v>2.83</v>
       </c>
-      <c r="G77" s="9">
+      <c r="G77" s="7">
         <v>0.02</v>
       </c>
-      <c r="H77" s="9">
+      <c r="H77" s="7">
         <v>0.77</v>
       </c>
-      <c r="I77" s="10">
+      <c r="I77" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>0.79</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A78" s="11">
+      <c r="A78" s="9">
         <v>44746</v>
       </c>
-      <c r="B78" s="3" t="s">
+      <c r="B78" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C78" s="3" t="s">
+      <c r="C78" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D78" s="3" t="s">
+      <c r="D78" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E78" s="3" t="s">
+      <c r="E78" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F78" s="3">
+      <c r="F78" s="1">
         <v>2.3199999999999998</v>
       </c>
-      <c r="G78" s="3">
+      <c r="G78" s="1">
         <v>4.3600000000000003</v>
       </c>
-      <c r="H78" s="3">
+      <c r="H78" s="1">
         <v>0.41</v>
       </c>
-      <c r="I78" s="10">
+      <c r="I78" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>4.7700000000000005</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A79" s="8">
+      <c r="A79" s="6">
         <v>44741</v>
       </c>
-      <c r="B79" s="9" t="s">
+      <c r="B79" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="C79" s="9" t="s">
+      <c r="C79" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D79" s="9" t="s">
+      <c r="D79" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E79" s="9" t="s">
+      <c r="E79" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F79" s="9">
+      <c r="F79" s="7">
         <v>1.88</v>
       </c>
-      <c r="G79" s="9">
+      <c r="G79" s="7">
         <v>1.98</v>
       </c>
-      <c r="H79" s="9">
+      <c r="H79" s="7">
         <v>0.7</v>
       </c>
-      <c r="I79" s="10">
+      <c r="I79" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.6799999999999997</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A80" s="11">
+      <c r="A80" s="9">
         <v>44745</v>
       </c>
-      <c r="B80" s="3" t="s">
+      <c r="B80" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C80" s="3" t="s">
+      <c r="C80" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D80" s="3" t="s">
+      <c r="D80" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E80" s="3" t="s">
+      <c r="E80" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="F80" s="3">
+      <c r="F80" s="1">
         <v>2.86</v>
       </c>
-      <c r="G80" s="3">
+      <c r="G80" s="1">
         <v>0.1</v>
       </c>
-      <c r="H80" s="3">
+      <c r="H80" s="1">
         <v>0.85</v>
       </c>
-      <c r="I80" s="10">
+      <c r="I80" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>0.95</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A81" s="8">
+      <c r="A81" s="6">
         <v>44726</v>
       </c>
-      <c r="B81" s="9" t="s">
+      <c r="B81" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="C81" s="9" t="s">
+      <c r="C81" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D81" s="9" t="s">
+      <c r="D81" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E81" s="9" t="s">
+      <c r="E81" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F81" s="9">
+      <c r="F81" s="7">
         <v>1.24</v>
       </c>
-      <c r="G81" s="9">
+      <c r="G81" s="7">
         <v>3.81</v>
       </c>
-      <c r="H81" s="9">
+      <c r="H81" s="7">
         <v>0.18</v>
       </c>
-      <c r="I81" s="10">
+      <c r="I81" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>3.99</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A82" s="11">
+      <c r="A82" s="9">
         <v>44738</v>
       </c>
-      <c r="B82" s="3" t="s">
+      <c r="B82" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="C82" s="3" t="s">
+      <c r="C82" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D82" s="3" t="s">
+      <c r="D82" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E82" s="3" t="s">
+      <c r="E82" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F82" s="3">
+      <c r="F82" s="1">
         <v>1.53</v>
       </c>
-      <c r="G82" s="3">
+      <c r="G82" s="1">
         <v>0.05</v>
       </c>
-      <c r="H82" s="3">
+      <c r="H82" s="1">
         <v>0.08</v>
       </c>
-      <c r="I82" s="10">
+      <c r="I82" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>0.13</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A83" s="8">
+      <c r="A83" s="6">
         <v>44744</v>
       </c>
-      <c r="B83" s="9" t="s">
+      <c r="B83" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="C83" s="9" t="s">
+      <c r="C83" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D83" s="9" t="s">
+      <c r="D83" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E83" s="9" t="s">
+      <c r="E83" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F83" s="9">
+      <c r="F83" s="7">
         <v>3.53</v>
       </c>
-      <c r="G83" s="9">
+      <c r="G83" s="7">
         <v>2.4900000000000002</v>
       </c>
-      <c r="H83" s="9">
+      <c r="H83" s="7">
         <v>0.68</v>
       </c>
-      <c r="I83" s="10">
+      <c r="I83" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>3.1700000000000004</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A84" s="11">
+      <c r="A84" s="9">
         <v>44749</v>
       </c>
-      <c r="B84" s="3" t="s">
+      <c r="B84" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="C84" s="3" t="s">
+      <c r="C84" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D84" s="3" t="s">
+      <c r="D84" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E84" s="3" t="s">
+      <c r="E84" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="F84" s="3">
+      <c r="F84" s="1">
         <v>6.06</v>
       </c>
-      <c r="G84" s="3">
+      <c r="G84" s="1">
         <v>0.06</v>
       </c>
-      <c r="H84" s="3">
+      <c r="H84" s="1">
         <v>1.26</v>
       </c>
-      <c r="I84" s="10">
+      <c r="I84" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.32</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A85" s="8">
+      <c r="A85" s="6">
         <v>44741</v>
       </c>
-      <c r="B85" s="9" t="s">
+      <c r="B85" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="C85" s="9" t="s">
+      <c r="C85" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D85" s="9" t="s">
+      <c r="D85" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E85" s="9" t="s">
+      <c r="E85" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F85" s="9">
+      <c r="F85" s="7">
         <v>2.2999999999999998</v>
       </c>
-      <c r="G85" s="9">
+      <c r="G85" s="7">
         <v>1.58</v>
       </c>
-      <c r="H85" s="9">
+      <c r="H85" s="7">
         <v>0.73</v>
       </c>
-      <c r="I85" s="10">
+      <c r="I85" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.31</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A86" s="11">
+      <c r="A86" s="9">
         <v>44746</v>
       </c>
-      <c r="B86" s="3" t="s">
+      <c r="B86" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C86" s="3" t="s">
+      <c r="C86" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D86" s="3" t="s">
+      <c r="D86" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E86" s="3" t="s">
+      <c r="E86" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F86" s="3">
+      <c r="F86" s="1">
         <v>1.86</v>
       </c>
-      <c r="G86" s="3">
+      <c r="G86" s="1">
         <v>3.14</v>
       </c>
-      <c r="H86" s="3">
+      <c r="H86" s="1">
         <v>0.43</v>
       </c>
-      <c r="I86" s="10">
+      <c r="I86" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>3.5700000000000003</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A87" s="8">
+      <c r="A87" s="6">
         <v>44746</v>
       </c>
-      <c r="B87" s="9" t="s">
+      <c r="B87" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="C87" s="9" t="s">
+      <c r="C87" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D87" s="9" t="s">
+      <c r="D87" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E87" s="9" t="s">
+      <c r="E87" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="F87" s="9">
+      <c r="F87" s="7">
         <v>5.05</v>
       </c>
-      <c r="G87" s="9">
+      <c r="G87" s="7">
         <v>0.13</v>
       </c>
-      <c r="H87" s="9">
+      <c r="H87" s="7">
         <v>2.0099999999999998</v>
       </c>
-      <c r="I87" s="10">
+      <c r="I87" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.1399999999999997</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A88" s="11">
+      <c r="A88" s="9">
         <v>44743</v>
       </c>
-      <c r="B88" s="3" t="s">
+      <c r="B88" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C88" s="3" t="s">
+      <c r="C88" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D88" s="3" t="s">
+      <c r="D88" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E88" s="3" t="s">
+      <c r="E88" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="F88" s="3">
+      <c r="F88" s="1">
         <v>6.42</v>
       </c>
-      <c r="G88" s="3">
+      <c r="G88" s="1">
         <v>0</v>
       </c>
-      <c r="H88" s="3">
+      <c r="H88" s="1">
         <v>0.71</v>
       </c>
-      <c r="I88" s="10">
+      <c r="I88" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>0.71</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A89" s="8">
+      <c r="A89" s="6">
         <v>44731</v>
       </c>
-      <c r="B89" s="9" t="s">
+      <c r="B89" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="C89" s="9" t="s">
+      <c r="C89" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="D89" s="9" t="s">
+      <c r="D89" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E89" s="9" t="s">
+      <c r="E89" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F89" s="9">
+      <c r="F89" s="7">
         <v>2.0099999999999998</v>
       </c>
-      <c r="G89" s="9">
+      <c r="G89" s="7">
         <v>0.13</v>
       </c>
-      <c r="H89" s="9">
+      <c r="H89" s="7">
         <v>0.15</v>
       </c>
-      <c r="I89" s="10">
+      <c r="I89" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>0.28000000000000003</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A90" s="11">
+      <c r="A90" s="9">
         <v>44741</v>
       </c>
-      <c r="B90" s="3" t="s">
+      <c r="B90" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C90" s="3" t="s">
+      <c r="C90" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D90" s="3" t="s">
+      <c r="D90" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E90" s="3" t="s">
+      <c r="E90" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F90" s="3">
+      <c r="F90" s="1">
         <v>3.9</v>
       </c>
-      <c r="G90" s="3">
+      <c r="G90" s="1">
         <v>0.66</v>
       </c>
-      <c r="H90" s="3">
+      <c r="H90" s="1">
         <v>0.91</v>
       </c>
-      <c r="I90" s="10">
+      <c r="I90" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.57</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A91" s="8">
+      <c r="A91" s="6">
         <v>44735</v>
       </c>
-      <c r="B91" s="9" t="s">
+      <c r="B91" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="C91" s="9" t="s">
+      <c r="C91" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D91" s="9" t="s">
+      <c r="D91" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E91" s="9" t="s">
+      <c r="E91" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F91" s="9">
+      <c r="F91" s="7">
         <v>2.0699999999999998</v>
       </c>
-      <c r="G91" s="9">
+      <c r="G91" s="7">
         <v>2.73</v>
       </c>
-      <c r="H91" s="9">
+      <c r="H91" s="7">
         <v>0.33</v>
       </c>
-      <c r="I91" s="10">
+      <c r="I91" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>3.06</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A92" s="11">
+      <c r="A92" s="9">
         <v>44733</v>
       </c>
-      <c r="B92" s="3" t="s">
+      <c r="B92" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="C92" s="3" t="s">
+      <c r="C92" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="D92" s="3" t="s">
+      <c r="D92" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E92" s="3" t="s">
+      <c r="E92" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F92" s="3">
+      <c r="F92" s="1">
         <v>1.72</v>
       </c>
-      <c r="G92" s="3">
+      <c r="G92" s="1">
         <v>3.63</v>
       </c>
-      <c r="H92" s="3">
+      <c r="H92" s="1">
         <v>0.23</v>
       </c>
-      <c r="I92" s="10">
+      <c r="I92" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>3.86</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A93" s="8">
+      <c r="A93" s="6">
         <v>44742</v>
       </c>
-      <c r="B93" s="9" t="s">
+      <c r="B93" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="C93" s="9" t="s">
+      <c r="C93" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D93" s="9" t="s">
+      <c r="D93" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E93" s="9" t="s">
+      <c r="E93" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F93" s="9">
+      <c r="F93" s="7">
         <v>1.78</v>
       </c>
-      <c r="G93" s="9">
+      <c r="G93" s="7">
         <v>2.69</v>
       </c>
-      <c r="H93" s="9">
+      <c r="H93" s="7">
         <v>0.55000000000000004</v>
       </c>
-      <c r="I93" s="10">
+      <c r="I93" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>3.24</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A94" s="11">
+      <c r="A94" s="9">
         <v>44716</v>
       </c>
-      <c r="B94" s="3" t="s">
+      <c r="B94" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="C94" s="3">
+      <c r="C94" s="1">
         <v>2600</v>
       </c>
-      <c r="D94" s="3" t="s">
+      <c r="D94" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E94" s="3" t="s">
+      <c r="E94" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="F94" s="3">
+      <c r="F94" s="1">
         <v>0.45</v>
       </c>
-      <c r="G94" s="3">
+      <c r="G94" s="1">
         <v>0</v>
       </c>
-      <c r="H94" s="3">
+      <c r="H94" s="1">
         <v>0.08</v>
       </c>
-      <c r="I94" s="10">
+      <c r="I94" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>0.08</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A95" s="8">
+      <c r="A95" s="6">
         <v>44739</v>
       </c>
-      <c r="B95" s="9" t="s">
+      <c r="B95" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="C95" s="9" t="s">
+      <c r="C95" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="D95" s="9" t="s">
+      <c r="D95" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E95" s="9" t="s">
+      <c r="E95" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="F95" s="9">
+      <c r="F95" s="7">
         <v>2.83</v>
       </c>
-      <c r="G95" s="9">
+      <c r="G95" s="7">
         <v>0.24</v>
       </c>
-      <c r="H95" s="9">
+      <c r="H95" s="7">
         <v>1.75</v>
       </c>
-      <c r="I95" s="10">
+      <c r="I95" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.99</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A96" s="11">
+      <c r="A96" s="9">
         <v>44744</v>
       </c>
-      <c r="B96" s="3" t="s">
+      <c r="B96" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="C96" s="3" t="s">
+      <c r="C96" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D96" s="3" t="s">
+      <c r="D96" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E96" s="3" t="s">
+      <c r="E96" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F96" s="3">
+      <c r="F96" s="1">
         <v>2.42</v>
       </c>
-      <c r="G96" s="3">
+      <c r="G96" s="1">
         <v>0.98</v>
       </c>
-      <c r="H96" s="3">
+      <c r="H96" s="1">
         <v>0.64</v>
       </c>
-      <c r="I96" s="10">
+      <c r="I96" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.62</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A97" s="8">
+      <c r="A97" s="6">
         <v>44749</v>
       </c>
-      <c r="B97" s="9" t="s">
+      <c r="B97" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="C97" s="9" t="s">
+      <c r="C97" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="D97" s="9" t="s">
+      <c r="D97" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E97" s="9" t="s">
+      <c r="E97" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="F97" s="9">
+      <c r="F97" s="7">
         <v>3.29</v>
       </c>
-      <c r="G97" s="9">
+      <c r="G97" s="7">
         <v>0.22</v>
       </c>
-      <c r="H97" s="9">
+      <c r="H97" s="7">
         <v>1.23</v>
       </c>
-      <c r="I97" s="10">
+      <c r="I97" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.45</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A98" s="11">
+      <c r="A98" s="9">
         <v>44732</v>
       </c>
-      <c r="B98" s="3" t="s">
+      <c r="B98" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="C98" s="3" t="s">
+      <c r="C98" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D98" s="3" t="s">
+      <c r="D98" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E98" s="3" t="s">
+      <c r="E98" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F98" s="3">
+      <c r="F98" s="1">
         <v>1.89</v>
       </c>
-      <c r="G98" s="3">
+      <c r="G98" s="1">
         <v>1.45</v>
       </c>
-      <c r="H98" s="3">
+      <c r="H98" s="1">
         <v>0.16</v>
       </c>
-      <c r="I98" s="10">
+      <c r="I98" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.6099999999999999</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A99" s="8">
+      <c r="A99" s="6">
         <v>44748</v>
       </c>
-      <c r="B99" s="9" t="s">
+      <c r="B99" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="C99" s="9" t="s">
+      <c r="C99" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="D99" s="9" t="s">
+      <c r="D99" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E99" s="9" t="s">
+      <c r="E99" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F99" s="9">
+      <c r="F99" s="7">
         <v>3.3</v>
       </c>
-      <c r="G99" s="9">
+      <c r="G99" s="7">
         <v>0.14000000000000001</v>
       </c>
-      <c r="H99" s="9">
+      <c r="H99" s="7">
         <v>1.37</v>
       </c>
-      <c r="I99" s="10">
+      <c r="I99" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.5100000000000002</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A100" s="11">
+      <c r="A100" s="9">
         <v>44731</v>
       </c>
-      <c r="B100" s="3" t="s">
+      <c r="B100" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="C100" s="3" t="s">
+      <c r="C100" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="D100" s="3" t="s">
+      <c r="D100" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E100" s="3" t="s">
+      <c r="E100" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F100" s="3">
+      <c r="F100" s="1">
         <v>2.17</v>
       </c>
-      <c r="G100" s="3">
+      <c r="G100" s="1">
         <v>1.31</v>
       </c>
-      <c r="H100" s="3">
+      <c r="H100" s="1">
         <v>0.31</v>
       </c>
-      <c r="I100" s="10">
+      <c r="I100" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>1.62</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A101" s="8">
+      <c r="A101" s="6">
         <v>44722</v>
       </c>
-      <c r="B101" s="9" t="s">
+      <c r="B101" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="C101" s="9" t="s">
+      <c r="C101" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D101" s="9" t="s">
+      <c r="D101" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E101" s="9" t="s">
+      <c r="E101" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F101" s="9">
+      <c r="F101" s="7">
         <v>1.18</v>
       </c>
-      <c r="G101" s="9">
+      <c r="G101" s="7">
         <v>0.7</v>
       </c>
-      <c r="H101" s="9">
+      <c r="H101" s="7">
         <v>0.19</v>
       </c>
-      <c r="I101" s="10">
+      <c r="I101" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>0.8899999999999999</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A102" s="11">
+      <c r="A102" s="9">
         <v>44748</v>
       </c>
-      <c r="B102" s="3" t="s">
+      <c r="B102" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="C102" s="3" t="s">
+      <c r="C102" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D102" s="3" t="s">
+      <c r="D102" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E102" s="3" t="s">
+      <c r="E102" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F102" s="3">
+      <c r="F102" s="1">
         <v>1.35</v>
       </c>
-      <c r="G102" s="3">
+      <c r="G102" s="1">
         <v>2.42</v>
       </c>
-      <c r="H102" s="3">
+      <c r="H102" s="1">
         <v>0.43</v>
       </c>
-      <c r="I102" s="10">
+      <c r="I102" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>2.85</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A103" s="12">
+      <c r="A103" s="10">
         <v>44742</v>
       </c>
-      <c r="B103" s="13" t="s">
+      <c r="B103" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="C103" s="13" t="s">
+      <c r="C103" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="D103" s="13" t="s">
+      <c r="D103" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="E103" s="13" t="s">
+      <c r="E103" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="F103" s="13">
+      <c r="F103" s="11">
         <v>1.9</v>
       </c>
-      <c r="G103" s="13">
+      <c r="G103" s="11">
         <v>0</v>
       </c>
-      <c r="H103" s="13">
+      <c r="H103" s="11">
         <v>0.69</v>
       </c>
-      <c r="I103" s="10">
+      <c r="I103" s="8">
         <f>Tabla4[[#This Row],[EU Sales]]+Tabla4[[#This Row],[Sales USA]]</f>
         <v>0.69</v>
       </c>
@@ -68312,14 +68398,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -68327,22 +68413,22 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="2" t="s">
         <v>145</v>
       </c>
     </row>
@@ -68476,32 +68562,102 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{511BB91C-9FF2-48C4-82D6-39AB8A600B14}">
-  <dimension ref="A3:A6"/>
+  <dimension ref="A3:C20"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="34.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>160</v>
-      </c>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="14"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="16"/>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>162</v>
-      </c>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="17"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="19"/>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>163</v>
-      </c>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="17"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="19"/>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>161</v>
-      </c>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="17"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="19"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="17"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="19"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="17"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="19"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="17"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="19"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="17"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="19"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="17"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="19"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="17"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="19"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="17"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="19"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="17"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="19"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="17"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="19"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="17"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="19"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="17"/>
+      <c r="B17" s="18"/>
+      <c r="C17" s="19"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="17"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="19"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="17"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="19"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="20"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="22"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>